<commit_message>
Fix sort issue in dononr pick table xlsx, add version with tissue inventory notes from Svitlana
</commit_message>
<xml_diff>
--- a/processed-data/21_Xenium/04_xenium_donors/xenium_donor_picks.xlsx
+++ b/processed-data/21_Xenium/04_xenium_donors/xenium_donor_picks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lieberinstitute-my.sharepoint.com/personal/louise_huuki_libd_org/Documents/LIBD_code/LFF_spatial_ERC/processed-data/21_Xenium/04_xenium_donors/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{AD6167BE-8ADE-CE4A-A413-A289664FF6BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C5A90094-9B3F-BC41-B6AE-B6B5C3F37C82}"/>
+  <xr:revisionPtr revIDLastSave="20" documentId="8_{AD6167BE-8ADE-CE4A-A413-A289664FF6BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D59C1D5B-61F6-9045-A48A-75C37306A799}"/>
   <bookViews>
     <workbookView xWindow="1500" yWindow="1400" windowWidth="27640" windowHeight="16680" xr2:uid="{516D38BB-D242-7945-94E2-0EDD02C8CBFA}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="xenium_donor_picks" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">xenium_donor_picks!$A$1:$L$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">xenium_donor_picks!$A$1:$M$1</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
@@ -699,6 +699,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1137,6 +1141,9 @@
       <c r="L3" t="s">
         <v>38</v>
       </c>
+      <c r="M3" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
@@ -1175,9 +1182,6 @@
       <c r="L4" t="s">
         <v>37</v>
       </c>
-      <c r="M4" t="s">
-        <v>39</v>
-      </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
@@ -1254,9 +1258,6 @@
       <c r="L6" t="s">
         <v>37</v>
       </c>
-      <c r="M6" t="s">
-        <v>41</v>
-      </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
@@ -1295,9 +1296,6 @@
       <c r="L7" t="s">
         <v>37</v>
       </c>
-      <c r="M7" t="s">
-        <v>42</v>
-      </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
@@ -1336,6 +1334,9 @@
       <c r="L8" t="s">
         <v>38</v>
       </c>
+      <c r="M8" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
@@ -1564,6 +1565,9 @@
       <c r="L14" t="s">
         <v>40</v>
       </c>
+      <c r="M14" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
@@ -1680,11 +1684,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L17" xr:uid="{6C4EF1EA-A7AD-C74F-86EA-F1C14CDD47D7}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L17">
-      <sortCondition ref="B1:B17"/>
-    </sortState>
-  </autoFilter>
+  <autoFilter ref="A1:M1" xr:uid="{6C4EF1EA-A7AD-C74F-86EA-F1C14CDD47D7}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>